<commit_message>
docs(entrega-2): corrige los casos CP-DEU-001, 003 y 011 y los vuelve a ejecutar
En la primera corrida quedaron en DUDA por pasos que faltaban o estaban mal
ordenados: no pedían elegir una cuenta (sin cuenta «Guardar gasto» queda
deshabilitado) y el 003 fijaba el tipo de cambio antes de cambiar la fecha a
otro mes, que la app descarta a propósito. Se agregan los pasos (elegir
«Efectivo» y, en el 003, volver al paso 1 para cargar de nuevo el tipo de
cambio) y se vuelven a ejecutar: PASSED.

Se actualizan casos/deu.md, 04, 06, README y los Excel: 197 casos con
resultado (183 PASSED, 9 FAILED, 1 DUDA, 4 BLOCKED).

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/entrega-2/06-reporte-de-ejecucion.xlsx
+++ b/entrega-2/06-reporte-de-ejecucion.xlsx
@@ -585,7 +585,7 @@
       </c>
       <c r="F3" s="4" t="inlineStr">
         <is>
-          <t>DUDA</t>
+          <t>PASSED</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
@@ -661,7 +661,7 @@
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>DUDA</t>
+          <t>PASSED</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
@@ -965,7 +965,7 @@
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>DUDA</t>
+          <t>PASSED</t>
         </is>
       </c>
       <c r="G13" s="3" t="inlineStr">
@@ -8119,7 +8119,7 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>183</t>
         </is>
       </c>
     </row>
@@ -8143,7 +8143,7 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -8191,7 +8191,7 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>93 %</t>
+          <t>95 %</t>
         </is>
       </c>
     </row>
@@ -8289,7 +8289,7 @@
       </c>
       <c r="C217" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="D217" t="inlineStr">
@@ -8299,7 +8299,7 @@
       </c>
       <c r="E217" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="F217" t="inlineStr">
@@ -8779,7 +8779,7 @@
       </c>
       <c r="C233" t="inlineStr">
         <is>
-          <t>112</t>
+          <t>115</t>
         </is>
       </c>
       <c r="D233" t="inlineStr">
@@ -8789,7 +8789,7 @@
       </c>
       <c r="E233" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="F233" t="inlineStr">

</xml_diff>

<commit_message>
docs(entrega-2): casos de Resumen por categoría (CP-CAT-001 a 006) y su ejecución
US-72 (torta por categoría) y US-73 (detalle de categoría) están implementadas
y no tenían casos. Se agregan 6 casos simples en casos/cat.md: la torta con una
porción por categoría, sin ingresos ni gastos eliminados y con «Resto» a partir
de 7 categorías; y el detalle de una categoría, su navegación por mes y hacia el
Resumen y el aviso de una categoría que no existe. US-84 no lleva casos porque
la función no existe.

Se ejecutaron con Playwright contra Vite + Supabase local: los 6 pasan. Se
actualizan 04, 06, README, la tabla de historias y los Excel: 203 casos con
resultado (189 PASSED, 9 FAILED, 1 DUDA, 4 BLOCKED).

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/entrega-2/06-reporte-de-ejecucion.xlsx
+++ b/entrega-2/06-reporte-de-ejecucion.xlsx
@@ -495,7 +495,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H251"/>
+  <dimension ref="A1:H258"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -8079,439 +8079,445 @@
         </is>
       </c>
     </row>
-    <row r="200"/>
+    <row r="200">
+      <c r="A200" s="3" t="inlineStr">
+        <is>
+          <t>CP-CAT-001</t>
+        </is>
+      </c>
+      <c r="B200" s="3" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="C200" s="3" t="inlineStr">
+        <is>
+          <t>La torta muestra una porción por categoría, con su monto y su porcentaje</t>
+        </is>
+      </c>
+      <c r="D200" s="3" t="inlineStr">
+        <is>
+          <t>US-72</t>
+        </is>
+      </c>
+      <c r="E200" s="3" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="F200" s="8" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="G200" s="3" t="inlineStr">
+        <is>
+          <t>Claude Code</t>
+        </is>
+      </c>
+      <c r="H200" s="3" t="n"/>
+    </row>
     <row r="201">
-      <c r="A201" s="9" t="inlineStr">
+      <c r="A201" s="3" t="inlineStr">
+        <is>
+          <t>CP-CAT-002</t>
+        </is>
+      </c>
+      <c r="B201" s="3" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="C201" s="3" t="inlineStr">
+        <is>
+          <t>Los ingresos y los gastos eliminados no entran en la torta</t>
+        </is>
+      </c>
+      <c r="D201" s="3" t="inlineStr">
+        <is>
+          <t>US-72</t>
+        </is>
+      </c>
+      <c r="E201" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F201" s="8" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="G201" s="3" t="inlineStr">
+        <is>
+          <t>Claude Code</t>
+        </is>
+      </c>
+      <c r="H201" s="3" t="n"/>
+    </row>
+    <row r="202">
+      <c r="A202" s="3" t="inlineStr">
+        <is>
+          <t>CP-CAT-003</t>
+        </is>
+      </c>
+      <c r="B202" s="3" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="C202" s="3" t="inlineStr">
+        <is>
+          <t>Con 7 categorías, las dos más chicas se agrupan en «Resto» en la torta</t>
+        </is>
+      </c>
+      <c r="D202" s="3" t="inlineStr">
+        <is>
+          <t>US-72</t>
+        </is>
+      </c>
+      <c r="E202" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F202" s="8" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="G202" s="3" t="inlineStr">
+        <is>
+          <t>Claude Code</t>
+        </is>
+      </c>
+      <c r="H202" s="3" t="n"/>
+    </row>
+    <row r="203">
+      <c r="A203" s="3" t="inlineStr">
+        <is>
+          <t>CP-CAT-004</t>
+        </is>
+      </c>
+      <c r="B203" s="3" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="C203" s="3" t="inlineStr">
+        <is>
+          <t>Tocar una categoría del Resumen abre su detalle del mes</t>
+        </is>
+      </c>
+      <c r="D203" s="3" t="inlineStr">
+        <is>
+          <t>US-73</t>
+        </is>
+      </c>
+      <c r="E203" s="3" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="F203" s="8" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="G203" s="3" t="inlineStr">
+        <is>
+          <t>Claude Code</t>
+        </is>
+      </c>
+      <c r="H203" s="3" t="n"/>
+    </row>
+    <row r="204">
+      <c r="A204" s="3" t="inlineStr">
+        <is>
+          <t>CP-CAT-005</t>
+        </is>
+      </c>
+      <c r="B204" s="3" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="C204" s="3" t="inlineStr">
+        <is>
+          <t>En el detalle, «Mes anterior» y «‹ Resumen» conservan la categoría y el mes</t>
+        </is>
+      </c>
+      <c r="D204" s="3" t="inlineStr">
+        <is>
+          <t>US-73</t>
+        </is>
+      </c>
+      <c r="E204" s="3" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="F204" s="8" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="G204" s="3" t="inlineStr">
+        <is>
+          <t>Claude Code</t>
+        </is>
+      </c>
+      <c r="H204" s="3" t="n"/>
+    </row>
+    <row r="205">
+      <c r="A205" s="3" t="inlineStr">
+        <is>
+          <t>CP-CAT-006</t>
+        </is>
+      </c>
+      <c r="B205" s="3" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="C205" s="3" t="inlineStr">
+        <is>
+          <t>Una categoría que no existe muestra un aviso con salida al Resumen</t>
+        </is>
+      </c>
+      <c r="D205" s="3" t="inlineStr">
+        <is>
+          <t>US-73</t>
+        </is>
+      </c>
+      <c r="E205" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F205" s="8" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="G205" s="3" t="inlineStr">
+        <is>
+          <t>Claude Code</t>
+        </is>
+      </c>
+      <c r="H205" s="3" t="n"/>
+    </row>
+    <row r="206"/>
+    <row r="207">
+      <c r="A207" s="9" t="inlineStr">
         <is>
           <t>Resumen</t>
-        </is>
-      </c>
-    </row>
-    <row r="202">
-      <c r="A202" s="10" t="inlineStr">
-        <is>
-          <t>Planificados</t>
-        </is>
-      </c>
-      <c r="B202" t="inlineStr">
-        <is>
-          <t>197</t>
-        </is>
-      </c>
-    </row>
-    <row r="203">
-      <c r="A203" s="10" t="inlineStr">
-        <is>
-          <t>Ejecutados (PASSED + FAILED + DUDA)</t>
-        </is>
-      </c>
-      <c r="B203" t="inlineStr">
-        <is>
-          <t>193</t>
-        </is>
-      </c>
-    </row>
-    <row r="204">
-      <c r="A204" s="10" t="inlineStr">
-        <is>
-          <t>PASSED</t>
-        </is>
-      </c>
-      <c r="B204" t="inlineStr">
-        <is>
-          <t>183</t>
-        </is>
-      </c>
-    </row>
-    <row r="205">
-      <c r="A205" s="10" t="inlineStr">
-        <is>
-          <t>FAILED</t>
-        </is>
-      </c>
-      <c r="B205" t="inlineStr">
-        <is>
-          <t>9</t>
-        </is>
-      </c>
-    </row>
-    <row r="206">
-      <c r="A206" s="10" t="inlineStr">
-        <is>
-          <t>DUDA (pasa, con dudas)</t>
-        </is>
-      </c>
-      <c r="B206" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-    </row>
-    <row r="207">
-      <c r="A207" s="10" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
-        </is>
-      </c>
-      <c r="B207" t="inlineStr">
-        <is>
-          <t>4</t>
         </is>
       </c>
     </row>
     <row r="208">
       <c r="A208" s="10" t="inlineStr">
         <is>
-          <t>No ejecutados</t>
+          <t>Planificados</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>203</t>
         </is>
       </c>
     </row>
     <row r="209">
       <c r="A209" s="10" t="inlineStr">
         <is>
-          <t>% avance (ejecutados/planificados)</t>
+          <t>Ejecutados (PASSED + FAILED + DUDA)</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>98 %</t>
+          <t>199</t>
         </is>
       </c>
     </row>
     <row r="210">
       <c r="A210" s="10" t="inlineStr">
         <is>
-          <t>% aprobados sobre ejecutados</t>
+          <t>PASSED</t>
         </is>
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>95 %</t>
+          <t>189</t>
         </is>
       </c>
     </row>
     <row r="211">
       <c r="A211" s="10" t="inlineStr">
         <is>
-          <t>Ejecutados con IA (Claude Code)</t>
+          <t>FAILED</t>
         </is>
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>155</t>
+          <t>9</t>
         </is>
       </c>
     </row>
     <row r="212">
       <c r="A212" s="10" t="inlineStr">
         <is>
-          <t>Ejecutados a mano por el equipo</t>
+          <t>DUDA (pasa, con dudas)</t>
         </is>
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>1</t>
         </is>
       </c>
     </row>
     <row r="213">
       <c r="A213" s="10" t="inlineStr">
         <is>
-          <t>Informados «ok» por el equipo, sin repetir</t>
+          <t>BLOCKED</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>21</t>
-        </is>
-      </c>
-    </row>
-    <row r="214"/>
+          <t>4</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" s="10" t="inlineStr">
+        <is>
+          <t>No ejecutados</t>
+        </is>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
     <row r="215">
-      <c r="A215" s="9" t="inlineStr">
-        <is>
-          <t>Por módulo</t>
+      <c r="A215" s="10" t="inlineStr">
+        <is>
+          <t>% avance (ejecutados/planificados)</t>
+        </is>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>98 %</t>
         </is>
       </c>
     </row>
     <row r="216">
       <c r="A216" s="10" t="inlineStr">
         <is>
+          <t>% aprobados sobre ejecutados</t>
+        </is>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>95 %</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" s="10" t="inlineStr">
+        <is>
+          <t>Ejecutados con IA (Claude Code)</t>
+        </is>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>161</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" s="10" t="inlineStr">
+        <is>
+          <t>Ejecutados a mano por el equipo</t>
+        </is>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" s="10" t="inlineStr">
+        <is>
+          <t>Informados «ok» por el equipo, sin repetir</t>
+        </is>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+    </row>
+    <row r="220"/>
+    <row r="221">
+      <c r="A221" s="9" t="inlineStr">
+        <is>
+          <t>Por módulo</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" s="10" t="inlineStr">
+        <is>
           <t>Módulo</t>
         </is>
       </c>
-      <c r="B216" s="10" t="inlineStr">
+      <c r="B222" s="10" t="inlineStr">
         <is>
           <t>Casos</t>
         </is>
       </c>
-      <c r="C216" s="10" t="inlineStr">
-        <is>
-          <t>PASSED</t>
-        </is>
-      </c>
-      <c r="D216" s="10" t="inlineStr">
+      <c r="C222" s="10" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="D222" s="10" t="inlineStr">
         <is>
           <t>FAILED</t>
         </is>
       </c>
-      <c r="E216" s="10" t="inlineStr">
+      <c r="E222" s="10" t="inlineStr">
         <is>
           <t>DUDA</t>
         </is>
       </c>
-      <c r="F216" s="10" t="inlineStr">
+      <c r="F222" s="10" t="inlineStr">
         <is>
           <t>BLOCKED</t>
         </is>
       </c>
-      <c r="G216" s="10" t="inlineStr">
+      <c r="G222" s="10" t="inlineStr">
         <is>
           <t>No ejecutados</t>
-        </is>
-      </c>
-    </row>
-    <row r="217">
-      <c r="A217" t="inlineStr">
-        <is>
-          <t>DEU-H · Gasto compartido con una persona y tope de la deuda (US-34, US-36 y US-41; CP-DEU-001 a 004, 011 a 013 y 025; 8 casos ejecutados con IA)</t>
-        </is>
-      </c>
-      <c r="B217" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="C217" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="D217" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E217" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="F217" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="G217" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="218">
-      <c r="A218" t="inlineStr">
-        <is>
-          <t>DEU-A · Gasto compartido: validaciones de create_transaction (US-34, CP-DEU-005 a 010)</t>
-        </is>
-      </c>
-      <c r="B218" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="C218" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="D218" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="E218" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="F218" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G218" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="219">
-      <c r="A219" t="inlineStr">
-        <is>
-          <t>DEU-B · Listado, filtro por estado y acceso (US-37 y US-38, CP-DEU-040 a 045)</t>
-        </is>
-      </c>
-      <c r="B219" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="C219" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="D219" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="E219" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="F219" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G219" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="220">
-      <c r="A220" t="inlineStr">
-        <is>
-          <t>DEU-C · Saldar, volver a pendiente y filtro por dirección (US-39, US-40 y US-79, CP-DEU-046 a 054)</t>
-        </is>
-      </c>
-      <c r="B220" t="inlineStr">
-        <is>
-          <t>9</t>
-        </is>
-      </c>
-      <c r="C220" t="inlineStr">
-        <is>
-          <t>9</t>
-        </is>
-      </c>
-      <c r="D220" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="E220" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="F220" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G220" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="221">
-      <c r="A221" t="inlineStr">
-        <is>
-          <t>DEU-D · Compartir con varias personas (US-82, CP-DEU-055, 056 y 057)</t>
-        </is>
-      </c>
-      <c r="B221" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="C221" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="D221" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="E221" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="F221" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="G221" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="222">
-      <c r="A222" t="inlineStr">
-        <is>
-          <t>DEU-E · Neto de reembolsos en el Resumen (US-30, CP-DEU-058 a 061)</t>
-        </is>
-      </c>
-      <c r="B222" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="C222" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="D222" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="E222" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="F222" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G222" t="inlineStr">
-        <is>
-          <t>0</t>
         </is>
       </c>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>DEU-G · Lectura y baja de gastos compartidos, alta de deuda suelta y create_debt por API (US-35, US-36 y US-41; CP-DEU-015 a 035, 16 casos ejecutados con IA)</t>
+          <t>DEU-H · Gasto compartido con una persona y tope de la deuda (US-34, US-36 y US-41; CP-DEU-001 a 004, 011 a 013 y 025; 8 casos ejecutados con IA)</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>8</t>
         </is>
       </c>
       <c r="C223" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>5</t>
         </is>
       </c>
       <c r="D223" t="inlineStr">
@@ -8521,12 +8527,12 @@
       </c>
       <c r="E223" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="F223" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G223" t="inlineStr">
@@ -8538,17 +8544,17 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>NAV-69 · Barra de navegación (US-69)</t>
+          <t>DEU-A · Gasto compartido: validaciones de create_transaction (US-34, CP-DEU-005 a 010)</t>
         </is>
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>6</t>
         </is>
       </c>
       <c r="C224" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>6</t>
         </is>
       </c>
       <c r="D224" t="inlineStr">
@@ -8575,17 +8581,17 @@
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>NAV-70 · Aviso de guardado y reintento (US-70)</t>
+          <t>DEU-B · Listado, filtro por estado y acceso (US-37 y US-38, CP-DEU-040 a 045)</t>
         </is>
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>6</t>
         </is>
       </c>
       <c r="C225" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>6</t>
         </is>
       </c>
       <c r="D225" t="inlineStr">
@@ -8612,22 +8618,22 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>EXP · Exportar CSV (US-47, 31 casos)</t>
+          <t>DEU-C · Saldar, volver a pendiente y filtro por dirección (US-39, US-40 y US-79, CP-DEU-046 a 054)</t>
         </is>
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>31</t>
+          <t>9</t>
         </is>
       </c>
       <c r="C226" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>9</t>
         </is>
       </c>
       <c r="D226" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>0</t>
         </is>
       </c>
       <c r="E226" t="inlineStr">
@@ -8649,22 +8655,22 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>IMP · Importar Excel (US-74 a US-79, 41 casos)</t>
+          <t>DEU-D · Compartir con varias personas (US-82, CP-DEU-055, 056 y 057)</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>3</t>
         </is>
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>0</t>
         </is>
       </c>
       <c r="D227" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="E227" t="inlineStr">
@@ -8674,7 +8680,7 @@
       </c>
       <c r="F227" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G227" t="inlineStr">
@@ -8686,115 +8692,217 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>SUS · Suscripciones (US-52 a US-63 y US-75, 48 casos)</t>
+          <t>DEU-E · Neto de reembolsos en el Resumen (US-30, CP-DEU-058 a 061)</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>48</t>
+          <t>4</t>
         </is>
       </c>
       <c r="C228" t="inlineStr">
         <is>
-          <t>45</t>
+          <t>4</t>
         </is>
       </c>
       <c r="D228" t="inlineStr">
         <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E228" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F228" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G228" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>DEU-G · Lectura y baja de gastos compartidos, alta de deuda suelta y create_debt por API (US-35, US-36 y US-41; CP-DEU-015 a 035, 16 casos ejecutados con IA)</t>
+        </is>
+      </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="C229" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="D229" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E229" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F229" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G229" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>NAV-69 · Barra de navegación (US-69)</t>
+        </is>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C230" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="D230" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E230" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F230" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G230" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>NAV-70 · Aviso de guardado y reintento (US-70)</t>
+        </is>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="C231" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="D231" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E231" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F231" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G231" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>EXP · Exportar CSV (US-47, 31 casos)</t>
+        </is>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
+      </c>
+      <c r="C232" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="D232" t="inlineStr">
+        <is>
           <t>3</t>
         </is>
       </c>
-      <c r="E228" t="inlineStr">
+      <c r="E232" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="F228" t="inlineStr">
+      <c r="F232" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="G228" t="inlineStr">
+      <c r="G232" t="inlineStr">
         <is>
           <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="229"/>
-    <row r="230"/>
-    <row r="231">
-      <c r="A231" s="9" t="inlineStr">
-        <is>
-          <t>Por prioridad</t>
-        </is>
-      </c>
-    </row>
-    <row r="232">
-      <c r="A232" s="10" t="inlineStr">
-        <is>
-          <t>Prioridad</t>
-        </is>
-      </c>
-      <c r="B232" s="10" t="inlineStr">
-        <is>
-          <t>Casos</t>
-        </is>
-      </c>
-      <c r="C232" s="10" t="inlineStr">
-        <is>
-          <t>PASSED</t>
-        </is>
-      </c>
-      <c r="D232" s="10" t="inlineStr">
-        <is>
-          <t>FAILED</t>
-        </is>
-      </c>
-      <c r="E232" s="10" t="inlineStr">
-        <is>
-          <t>DUDA</t>
-        </is>
-      </c>
-      <c r="F232" s="10" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
-        </is>
-      </c>
-      <c r="G232" s="10" t="inlineStr">
-        <is>
-          <t>No ejecutados</t>
         </is>
       </c>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>IMP · Importar Excel (US-74 a US-79, 41 casos)</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>126</t>
+          <t>41</t>
         </is>
       </c>
       <c r="C233" t="inlineStr">
         <is>
-          <t>115</t>
+          <t>40</t>
         </is>
       </c>
       <c r="D233" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E233" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F233" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G233" t="inlineStr">
@@ -8806,22 +8914,22 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>SUS · Suscripciones (US-52 a US-63 y US-75, 48 casos)</t>
         </is>
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>67</t>
+          <t>48</t>
         </is>
       </c>
       <c r="C234" t="inlineStr">
         <is>
-          <t>65</t>
+          <t>45</t>
         </is>
       </c>
       <c r="D234" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E234" t="inlineStr">
@@ -8843,22 +8951,22 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>CAT · Resumen por categoría (US-72 y US-73, 6 casos)</t>
         </is>
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>6</t>
         </is>
       </c>
       <c r="C235" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>6</t>
         </is>
       </c>
       <c r="D235" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="E235" t="inlineStr">
@@ -8882,153 +8990,310 @@
     <row r="238">
       <c r="A238" s="9" t="inlineStr">
         <is>
-          <t>Defectos abiertos por severidad</t>
+          <t>Por prioridad</t>
         </is>
       </c>
     </row>
     <row r="239">
       <c r="A239" s="10" t="inlineStr">
         <is>
-          <t>Severidad</t>
+          <t>Prioridad</t>
         </is>
       </c>
       <c r="B239" s="10" t="inlineStr">
         <is>
-          <t>Abiertos</t>
+          <t>Casos</t>
         </is>
       </c>
       <c r="C239" s="10" t="inlineStr">
         <is>
-          <t>IDs</t>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="D239" s="10" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="E239" s="10" t="inlineStr">
+        <is>
+          <t>DUDA</t>
+        </is>
+      </c>
+      <c r="F239" s="10" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
+      <c r="G239" s="10" t="inlineStr">
+        <is>
+          <t>No ejecutados</t>
         </is>
       </c>
     </row>
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>Crítica</t>
-        </is>
-      </c>
-      <c r="B240" t="n">
-        <v>0</v>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>129</t>
+        </is>
       </c>
       <c r="C240" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>118</t>
+        </is>
+      </c>
+      <c r="D240" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="E240" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F240" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G240" t="inlineStr">
+        <is>
+          <t>0</t>
         </is>
       </c>
     </row>
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>Alta</t>
-        </is>
-      </c>
-      <c r="B241" t="n">
-        <v>0</v>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
       </c>
       <c r="C241" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>68</t>
+        </is>
+      </c>
+      <c r="D241" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E241" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F241" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G241" t="inlineStr">
+        <is>
+          <t>0</t>
         </is>
       </c>
     </row>
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="B242" t="n">
-        <v>4</v>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t>DEF-030, DEF-031, DEF-032, DEF-037</t>
-        </is>
-      </c>
-    </row>
-    <row r="243">
-      <c r="A243" t="inlineStr">
-        <is>
-          <t>Baja</t>
-        </is>
-      </c>
-      <c r="B243" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="C243" t="inlineStr">
-        <is>
-          <t>DEF-033, DEF-034, DEF-035, DEF-036</t>
-        </is>
-      </c>
-    </row>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D242" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E242" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F242" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G242" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="243"/>
     <row r="244"/>
-    <row r="245"/>
+    <row r="245">
+      <c r="A245" s="9" t="inlineStr">
+        <is>
+          <t>Defectos abiertos por severidad</t>
+        </is>
+      </c>
+    </row>
     <row r="246">
-      <c r="A246" s="9" t="inlineStr">
-        <is>
-          <t>Criterios de salida (docs/07-plan-de-testing.md §6)</t>
+      <c r="A246" s="10" t="inlineStr">
+        <is>
+          <t>Severidad</t>
+        </is>
+      </c>
+      <c r="B246" s="10" t="inlineStr">
+        <is>
+          <t>Abiertos</t>
+        </is>
+      </c>
+      <c r="C246" s="10" t="inlineStr">
+        <is>
+          <t>IDs</t>
         </is>
       </c>
     </row>
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>1. Cero defectos de severidad Crítica abiertos</t>
-        </is>
+          <t>Crítica</t>
+        </is>
+      </c>
+      <c r="B247" t="n">
+        <v>0</v>
       </c>
       <c r="C247" t="inlineStr">
         <is>
-          <t>Cumplido</t>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>2. Cero defectos de severidad Alta abiertos, o justificados por el PO</t>
-        </is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="B248" t="n">
+        <v>0</v>
       </c>
       <c r="C248" t="inlineStr">
         <is>
-          <t>Cumplido</t>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>3. Todos los casos de prioridad Alta ejecutados</t>
-        </is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="B249" t="n">
+        <v>4</v>
       </c>
       <c r="C249" t="inlineStr">
         <is>
-          <t>No cumplido: 122 de 126 casos de prioridad Alta ejecutados. No ejecutados: 4, todos BLOCKED porque dependen de una funcionalidad todavía no implementada: US-82 (issue #270), CP-DEU-055, 056, 057 y CP-DEU-013. Se ejecutan en V3.</t>
+          <t>DEF-030, DEF-031, DEF-032, DEF-037</t>
         </is>
       </c>
     </row>
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C250" t="inlineStr">
+        <is>
+          <t>DEF-033, DEF-034, DEF-035, DEF-036</t>
+        </is>
+      </c>
+    </row>
+    <row r="251"/>
+    <row r="252"/>
+    <row r="253">
+      <c r="A253" s="9" t="inlineStr">
+        <is>
+          <t>Criterios de salida (docs/07-plan-de-testing.md §6)</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>1. Cero defectos de severidad Crítica abiertos</t>
+        </is>
+      </c>
+      <c r="C254" t="inlineStr">
+        <is>
+          <t>Cumplido</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>2. Cero defectos de severidad Alta abiertos, o justificados por el PO</t>
+        </is>
+      </c>
+      <c r="C255" t="inlineStr">
+        <is>
+          <t>Cumplido</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="inlineStr">
+        <is>
+          <t>3. Todos los casos de prioridad Alta ejecutados</t>
+        </is>
+      </c>
+      <c r="C256" t="inlineStr">
+        <is>
+          <t>No cumplido: 125 de 129 casos de prioridad Alta ejecutados. No ejecutados: 4, todos BLOCKED porque dependen de una funcionalidad todavía no implementada: US-82 (issue #270), CP-DEU-055, 056, 057 y CP-DEU-013. Se ejecutan en V3.</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="inlineStr">
+        <is>
           <t>4. Toda invariante del alcance con al menos un caso ejecutado</t>
         </is>
       </c>
-      <c r="C250" t="inlineStr">
+      <c r="C257" t="inlineStr">
         <is>
           <t>Parcial</t>
         </is>
       </c>
     </row>
-    <row r="251">
-      <c r="A251" t="inlineStr">
+    <row r="258">
+      <c r="A258" t="inlineStr">
         <is>
           <t>5. Regresión de V1 ejecutada y defectos corregidos confirmados</t>
         </is>
       </c>
-      <c r="C251" t="inlineStr">
+      <c r="C258" t="inlineStr">
         <is>
           <t>No evaluado</t>
         </is>

</xml_diff>

<commit_message>
docs(entrega-2): el 06 apunta a los gráficos y la guía da por mergeada la regresión
Con el PR #310 en main, la guía ya no necesita aclarar dónde está la regresión. El 06 decía
que la planilla tenía un gráfico que no existía: ahora enlaza los SVG de graficos/. Importar
Excel cubre US-74, US-76, US-77 y US-78, no «US-74 a US-79» (US-79 es de Deudas).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/entrega-2/06-reporte-de-ejecucion.xlsx
+++ b/entrega-2/06-reporte-de-ejecucion.xlsx
@@ -8877,7 +8877,7 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>IMP · Importar Excel (US-74 a US-79, 41 casos)</t>
+          <t>IMP · Importar Excel (US-74, US-76, US-77 y US-78, 41 casos)</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
@@ -9299,6 +9299,8 @@
         </is>
       </c>
     </row>
+    <row r="259"/>
+    <row r="260"/>
     <row r="261">
       <c r="A261" s="9" t="inlineStr">
         <is>
@@ -11628,6 +11630,7 @@
       </c>
       <c r="H322" s="3" t="n"/>
     </row>
+    <row r="323"/>
     <row r="324">
       <c r="A324" s="9" t="inlineStr">
         <is>
@@ -11767,6 +11770,7 @@
         </is>
       </c>
     </row>
+    <row r="336"/>
     <row r="337">
       <c r="A337" s="9" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
docs(entrega-2): el equipo repasó a mano todos los casos después de la ejecución con Claude Code
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/entrega-2/06-reporte-de-ejecucion.xlsx
+++ b/entrega-2/06-reporte-de-ejecucion.xlsx
@@ -8307,7 +8307,6 @@
       </c>
       <c r="H205" s="3" t="n"/>
     </row>
-    <row r="206"/>
     <row r="207">
       <c r="A207" s="9" t="inlineStr">
         <is>
@@ -8459,7 +8458,6 @@
         </is>
       </c>
     </row>
-    <row r="220"/>
     <row r="221">
       <c r="A221" s="9" t="inlineStr">
         <is>
@@ -8985,8 +8983,6 @@
         </is>
       </c>
     </row>
-    <row r="236"/>
-    <row r="237"/>
     <row r="238">
       <c r="A238" s="9" t="inlineStr">
         <is>
@@ -9142,8 +9138,6 @@
         </is>
       </c>
     </row>
-    <row r="243"/>
-    <row r="244"/>
     <row r="245">
       <c r="A245" s="9" t="inlineStr">
         <is>
@@ -9230,8 +9224,6 @@
         </is>
       </c>
     </row>
-    <row r="251"/>
-    <row r="252"/>
     <row r="253">
       <c r="A253" s="9" t="inlineStr">
         <is>
@@ -9295,12 +9287,10 @@
       </c>
       <c r="C258" t="inlineStr">
         <is>
-          <t>Cumplido, con salvedades: Confirmación de defectos de V1 ejecutada el 2026-10-28: 18 confirmados corregidos en V2, 3 confirmados en parte (DEF-021, DEF-027 y DEF-028) y 1 no concluyente (DEF-023, de severidad Alta, cerrado por decisión del equipo; se reabre si reaparece). Regresión de los 60 casos de V1 seleccionados (`03`) ejecutada el 2026-10-28 con IA: 60 PASSED, sin defectos nuevos. Salvedades: todo se verificó en local (DEF-005 depende de la configuración de Auth del proyecto hosteado, que no se verificó) y el repaso manual de los 39 casos de prioridad Alta está pendiente.</t>
-        </is>
-      </c>
-    </row>
-    <row r="259"/>
-    <row r="260"/>
+          <t>Cumplido, con salvedades: Confirmación de defectos de V1 ejecutada el 2026-10-28: 18 confirmados corregidos en V2, 3 confirmados en parte (DEF-021, DEF-027 y DEF-028) y 1 no concluyente (DEF-023, de severidad Alta, cerrado por decisión del equipo; se reabre si reaparece). Regresión de los 60 casos de V1 seleccionados (`03`) ejecutada el 2026-10-28 con IA: 60 PASSED, sin defectos nuevos. Salvedades: todo se verificó en local (DEF-005 depende de la configuración de Auth del proyecto hosteado, que no se verificó) y el repaso manual del equipo no dejó capturas ni un resultado por caso.</t>
+        </is>
+      </c>
+    </row>
     <row r="261">
       <c r="A261" s="9" t="inlineStr">
         <is>
@@ -11630,7 +11620,6 @@
       </c>
       <c r="H322" s="3" t="n"/>
     </row>
-    <row r="323"/>
     <row r="324">
       <c r="A324" s="9" t="inlineStr">
         <is>
@@ -11749,12 +11738,12 @@
     <row r="334">
       <c r="A334" s="10" t="inlineStr">
         <is>
-          <t>Repasados a mano por el equipo (prioridad Alta)</t>
+          <t>Repasados a mano por el equipo</t>
         </is>
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t>pendiente (0 de 39)</t>
+          <t>60 de 60</t>
         </is>
       </c>
     </row>
@@ -11770,7 +11759,6 @@
         </is>
       </c>
     </row>
-    <row r="336"/>
     <row r="337">
       <c r="A337" s="9" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
docs(entrega-2): quién repasó a mano cada módulo después de la ejecución con Claude Code
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/entrega-2/06-reporte-de-ejecucion.xlsx
+++ b/entrega-2/06-reporte-de-ejecucion.xlsx
@@ -8458,6 +8458,18 @@
         </is>
       </c>
     </row>
+    <row r="220">
+      <c r="A220" s="10" t="inlineStr">
+        <is>
+          <t>Repaso manual posterior (después de Claude Code)</t>
+        </is>
+      </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>DEU: Mariana · NAV: Santiago · EXP: Joaquín · IMP: Valentina · SUS: Micaela · CAT y regresión de V1: el equipo</t>
+        </is>
+      </c>
+    </row>
     <row r="221">
       <c r="A221" s="9" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
docs(entrega-2): el repaso manual se hizo en el deploy y la regresión de V1 la ejecutó Joaquín
Después de la ejecución con Claude Code (local), el equipo repasó a mano los
casos de V2 en el deploy de Vercel, y Joaquín ejecutó a mano los 60 casos de
la regresión de V1 en el deploy. Se actualizan los .md y las planillas de
ejecución (04 y 06) y se saca la nota de que el repaso no dejó evidencia por caso.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/entrega-2/06-reporte-de-ejecucion.xlsx
+++ b/entrega-2/06-reporte-de-ejecucion.xlsx
@@ -8461,12 +8461,12 @@
     <row r="220">
       <c r="A220" s="10" t="inlineStr">
         <is>
-          <t>Repaso manual posterior (después de Claude Code)</t>
+          <t>Repaso manual posterior en el deploy (después de Claude Code)</t>
         </is>
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>DEU: Mariana · NAV: Santiago · EXP: Joaquín · IMP: Valentina · SUS: Micaela · CAT y regresión de V1: el equipo</t>
+          <t>DEU: Mariana · NAV: Santiago · EXP: Joaquín · IMP: Valentina · SUS: Micaela · CAT: el equipo · Regresión de V1: Joaquín</t>
         </is>
       </c>
     </row>
@@ -9299,7 +9299,7 @@
       </c>
       <c r="C258" t="inlineStr">
         <is>
-          <t>Cumplido, con salvedades: Confirmación de defectos de V1 ejecutada el 2026-10-28: 18 confirmados corregidos en V2, 3 confirmados en parte (DEF-021, DEF-027 y DEF-028) y 1 no concluyente (DEF-023, de severidad Alta, cerrado por decisión del equipo; se reabre si reaparece). Regresión de los 60 casos de V1 seleccionados (`03`) ejecutada el 2026-10-28 con IA: 60 PASSED, sin defectos nuevos. Salvedades: todo se verificó en local (DEF-005 depende de la configuración de Auth del proyecto hosteado, que no se verificó) y el repaso manual del equipo no dejó capturas ni un resultado por caso.</t>
+          <t>Cumplido, con salvedades: Confirmación de defectos de V1 ejecutada el 2026-10-28: 18 confirmados corregidos en V2, 3 confirmados en parte (DEF-021, DEF-027 y DEF-028) y 1 no concluyente (DEF-023, de severidad Alta, cerrado por decisión del equipo; se reabre si reaparece). Regresión de los 60 casos de V1 seleccionados (`03`) ejecutada el 2026-10-28 con IA: 60 PASSED, sin defectos nuevos. Salvedades: todo se verificó en local (DEF-005 depende de la configuración de Auth del proyecto hosteado, que no se verificó) y el repaso manual posterior se hizo en el deploy.</t>
         </is>
       </c>
     </row>
@@ -11750,7 +11750,7 @@
     <row r="334">
       <c r="A334" s="10" t="inlineStr">
         <is>
-          <t>Repasados a mano por el equipo</t>
+          <t>Ejecutados a mano por Joaquín en el deploy</t>
         </is>
       </c>
       <c r="B334" t="inlineStr">

</xml_diff>